<commit_message>
Apply Etsy-friendly aesthetic redesign to Budget Planner
Replace corporate green/blue palette with warm, feminine tones: dusty rose
headers, soft pink sections, mint green positive fills, warm cream backgrounds,
antique gold KPI highlights, and warm brown text throughout.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Ultimate Budget Planner.xlsx
+++ b/output/Ultimate Budget Planner.xlsx
@@ -60,7 +60,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,47 +71,46 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00212529"/>
+      <color rgb="004A3728"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="004A3728"/>
       <sz val="20"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00495057"/>
+      <color rgb="004A3728"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="004A3728"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00212529"/>
+      <color rgb="004A3728"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00495057"/>
+      <color rgb="004A3728"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002D6A4F"/>
+      <color rgb="00C9A84C"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00495057"/>
+      <color rgb="004A3728"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -120,23 +119,23 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00495057"/>
+      <color rgb="004A3728"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00495057"/>
+      <color rgb="004A3728"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002D6A4F"/>
+      <color rgb="00C9A84C"/>
       <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001B4F72"/>
+      <color rgb="004A3728"/>
       <sz val="12"/>
     </font>
     <font>
@@ -146,25 +145,26 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001B4F72"/>
+      <color rgb="001A7272"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="004A3728"/>
       <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00495057"/>
+      <color rgb="004A3728"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00212529"/>
+      <color rgb="004A3728"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00495057"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -174,47 +174,41 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00495057"/>
+      <color rgb="004A3728"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="002D6A4F"/>
+      <color rgb="001A7272"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002D6A4F"/>
+      <color rgb="001A7272"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="002D6A4F"/>
+      <color rgb="001A7272"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002D6A4F"/>
+      <color rgb="001A7272"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00212529"/>
+      <color rgb="004A3728"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00212529"/>
+      <color rgb="004A3728"/>
       <sz val="16"/>
     </font>
   </fonts>
@@ -227,17 +221,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D8F3DC"/>
+        <fgColor rgb="00D4EDEA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002D6A4F"/>
+        <fgColor rgb="00C9B8B8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B4F72"/>
+        <fgColor rgb="00E8D5D5"/>
       </patternFill>
     </fill>
     <fill>
@@ -247,7 +241,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8F9FA"/>
+        <fgColor rgb="00FDF6F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -275,13 +269,13 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </left>
       <right style="thin">
         <color rgb="00E9ECEF"/>
       </right>
       <top style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </top>
       <bottom style="thin">
         <color rgb="00E9ECEF"/>
@@ -295,7 +289,7 @@
         <color rgb="00E9ECEF"/>
       </right>
       <top style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </top>
       <bottom style="thin">
         <color rgb="00E9ECEF"/>
@@ -306,10 +300,10 @@
         <color rgb="00E9ECEF"/>
       </left>
       <right style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </right>
       <top style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </top>
       <bottom style="thin">
         <color rgb="00E9ECEF"/>
@@ -317,7 +311,7 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </left>
       <right style="thin">
         <color rgb="00E9ECEF"/>
@@ -334,7 +328,7 @@
         <color rgb="00E9ECEF"/>
       </left>
       <right style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </right>
       <top style="thin">
         <color rgb="00E9ECEF"/>
@@ -345,7 +339,7 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </left>
       <right style="thin">
         <color rgb="00E9ECEF"/>
@@ -354,7 +348,7 @@
         <color rgb="00E9ECEF"/>
       </top>
       <bottom style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </bottom>
     </border>
     <border>
@@ -368,7 +362,7 @@
         <color rgb="00E9ECEF"/>
       </top>
       <bottom style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </bottom>
     </border>
     <border>
@@ -376,13 +370,13 @@
         <color rgb="00E9ECEF"/>
       </left>
       <right style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </right>
       <top style="thin">
         <color rgb="00E9ECEF"/>
       </top>
       <bottom style="medium">
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </bottom>
     </border>
     <border>
@@ -436,16 +430,16 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -548,14 +542,14 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="9" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="9" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -573,13 +567,13 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="19" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -606,7 +600,7 @@
     <xf numFmtId="10" fontId="0" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -646,18 +640,18 @@
     <dxf>
       <font>
         <name val="Calibri"/>
-        <color rgb="002D6A4F"/>
+        <color rgb="001A7272"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00B7E4C7"/>
+          <fgColor rgb="00B2D8D8"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <name val="Calibri"/>
-        <color rgb="00E63946"/>
+        <color rgb="00D4756B"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -668,7 +662,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00B7E4C7"/>
+          <fgColor rgb="00B2D8D8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -682,7 +676,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00F4A261"/>
+          <fgColor rgb="00C9A84C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -724,7 +718,7 @@
       <font>
         <name val="Calibri"/>
         <b val="1"/>
-        <color rgb="00E63946"/>
+        <color rgb="00D4756B"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -737,7 +731,7 @@
         <name val="Calibri"/>
         <i val="1"/>
         <strike val="1"/>
-        <color rgb="00495057"/>
+        <color rgb="004A3728"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -2054,7 +2048,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="009D4EDD"/>
+    <tabColor rgb="00C9A84C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:H37"/>
@@ -2134,7 +2128,7 @@
         </is>
       </c>
       <c r="F5" s="83" t="n">
-        <v>46552</v>
+        <v>46553</v>
       </c>
       <c r="G5" s="82" t="inlineStr">
         <is>
@@ -2202,7 +2196,7 @@
         </is>
       </c>
       <c r="F10" s="83" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="G10" s="82" t="inlineStr">
         <is>
@@ -2270,7 +2264,7 @@
         </is>
       </c>
       <c r="F15" s="83" t="n">
-        <v>46917</v>
+        <v>46918</v>
       </c>
       <c r="G15" s="82" t="inlineStr">
         <is>
@@ -2338,7 +2332,7 @@
         </is>
       </c>
       <c r="F20" s="83" t="n">
-        <v>47282</v>
+        <v>47283</v>
       </c>
       <c r="G20" s="82" t="inlineStr">
         <is>
@@ -2406,7 +2400,7 @@
         </is>
       </c>
       <c r="F25" s="83" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="G25" s="82" t="inlineStr">
         <is>
@@ -2684,7 +2678,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00C9184A"/>
+    <tabColor rgb="00D4756B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:N19"/>
@@ -3308,7 +3302,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0040A5C9"/>
+    <tabColor rgb="00B2D8D8"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:I17"/>
@@ -3420,7 +3414,7 @@
         <v/>
       </c>
       <c r="I4" s="83" t="n">
-        <v>46387</v>
+        <v>46388</v>
       </c>
     </row>
     <row r="5">
@@ -3494,7 +3488,7 @@
         <v/>
       </c>
       <c r="I6" s="83" t="n">
-        <v>46487</v>
+        <v>46488</v>
       </c>
     </row>
     <row r="7">
@@ -3531,7 +3525,7 @@
         <v/>
       </c>
       <c r="I7" s="47" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="8">
@@ -3568,7 +3562,7 @@
         <v/>
       </c>
       <c r="I8" s="83" t="n">
-        <v>46367</v>
+        <v>46368</v>
       </c>
     </row>
     <row r="9">
@@ -3605,7 +3599,7 @@
         <v/>
       </c>
       <c r="I9" s="47" t="n">
-        <v>46337</v>
+        <v>46338</v>
       </c>
     </row>
     <row r="10">
@@ -3642,7 +3636,7 @@
         <v/>
       </c>
       <c r="I10" s="83" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="11">
@@ -3679,7 +3673,7 @@
         <v/>
       </c>
       <c r="I11" s="47" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
     </row>
     <row r="12">
@@ -3716,7 +3710,7 @@
         <v/>
       </c>
       <c r="I12" s="83" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="13">
@@ -3753,7 +3747,7 @@
         <v/>
       </c>
       <c r="I13" s="47" t="n">
-        <v>46387</v>
+        <v>46388</v>
       </c>
     </row>
     <row r="14">
@@ -3790,7 +3784,7 @@
         <v/>
       </c>
       <c r="I14" s="83" t="n">
-        <v>46437</v>
+        <v>46438</v>
       </c>
     </row>
     <row r="15">
@@ -3827,7 +3821,7 @@
         <v/>
       </c>
       <c r="I15" s="47" t="n">
-        <v>46367</v>
+        <v>46368</v>
       </c>
     </row>
     <row r="17">
@@ -3898,7 +3892,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="006C757D"/>
+    <tabColor rgb="00E8D5D5"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:H18"/>
@@ -3994,7 +3988,7 @@
         <v/>
       </c>
       <c r="F4" s="83" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="G4" s="22" t="inlineStr">
         <is>
@@ -4031,7 +4025,7 @@
         <v/>
       </c>
       <c r="F5" s="47" t="n">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="G5" s="48" t="inlineStr">
         <is>
@@ -4068,7 +4062,7 @@
         <v/>
       </c>
       <c r="F6" s="83" t="n">
-        <v>46387</v>
+        <v>46388</v>
       </c>
       <c r="G6" s="22" t="inlineStr">
         <is>
@@ -4105,7 +4099,7 @@
         <v/>
       </c>
       <c r="F7" s="47" t="n">
-        <v>46205</v>
+        <v>46206</v>
       </c>
       <c r="G7" s="48" t="inlineStr">
         <is>
@@ -4142,7 +4136,7 @@
         <v/>
       </c>
       <c r="F8" s="83" t="n">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="G8" s="22" t="inlineStr">
         <is>
@@ -4179,7 +4173,7 @@
         <v/>
       </c>
       <c r="F9" s="47" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="G9" s="48" t="inlineStr">
         <is>
@@ -4216,7 +4210,7 @@
         <v/>
       </c>
       <c r="F10" s="83" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="G10" s="22" t="inlineStr">
         <is>
@@ -4253,7 +4247,7 @@
         <v/>
       </c>
       <c r="F11" s="47" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
       <c r="G11" s="48" t="inlineStr">
         <is>
@@ -4290,7 +4284,7 @@
         <v/>
       </c>
       <c r="F12" s="83" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="G12" s="22" t="inlineStr">
         <is>
@@ -4327,7 +4321,7 @@
         <v/>
       </c>
       <c r="F13" s="47" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
       <c r="G13" s="48" t="inlineStr">
         <is>
@@ -4364,7 +4358,7 @@
         <v/>
       </c>
       <c r="F14" s="83" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="G14" s="22" t="inlineStr">
         <is>
@@ -4401,7 +4395,7 @@
         <v/>
       </c>
       <c r="F15" s="47" t="n">
-        <v>46437</v>
+        <v>46438</v>
       </c>
       <c r="G15" s="48" t="inlineStr">
         <is>
@@ -4499,7 +4493,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00F4A261"/>
+    <tabColor rgb="00C9A84C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:L21"/>
@@ -4637,7 +4631,7 @@
       </c>
       <c r="J4" s="22" t="n"/>
       <c r="K4" s="83" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L4" s="9">
         <f>IF(G4="Yes","✅ Paid",IF(I4&lt;0,"🔴 Overdue",IF(I4&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -4686,7 +4680,7 @@
       </c>
       <c r="J5" s="48" t="n"/>
       <c r="K5" s="47" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L5" s="12">
         <f>IF(G5="Yes","✅ Paid",IF(I5&lt;0,"🔴 Overdue",IF(I5&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -4782,7 +4776,7 @@
       </c>
       <c r="J7" s="48" t="n"/>
       <c r="K7" s="47" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L7" s="12">
         <f>IF(G7="Yes","✅ Paid",IF(I7&lt;0,"🔴 Overdue",IF(I7&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -4925,7 +4919,7 @@
       </c>
       <c r="J10" s="22" t="n"/>
       <c r="K10" s="83" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L10" s="9">
         <f>IF(G10="Yes","✅ Paid",IF(I10&lt;0,"🔴 Overdue",IF(I10&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -5115,7 +5109,7 @@
       </c>
       <c r="J14" s="22" t="n"/>
       <c r="K14" s="83" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L14" s="9">
         <f>IF(G14="Yes","✅ Paid",IF(I14&lt;0,"🔴 Overdue",IF(I14&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -5164,7 +5158,7 @@
       </c>
       <c r="J15" s="48" t="n"/>
       <c r="K15" s="47" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L15" s="12">
         <f>IF(G15="Yes","✅ Paid",IF(I15&lt;0,"🔴 Overdue",IF(I15&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -5260,7 +5254,7 @@
       </c>
       <c r="J17" s="48" t="n"/>
       <c r="K17" s="47" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L17" s="12">
         <f>IF(G17="Yes","✅ Paid",IF(I17&lt;0,"🔴 Overdue",IF(I17&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -5309,7 +5303,7 @@
       </c>
       <c r="J18" s="22" t="n"/>
       <c r="K18" s="83" t="n">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="L18" s="9">
         <f>IF(G18="Yes","✅ Paid",IF(I18&lt;0,"🔴 Overdue",IF(I18&lt;=3,"⚠️ Due Soon","📅 Upcoming")))</f>
@@ -5421,7 +5415,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001B4F72"/>
+    <tabColor rgb="00E8D5D5"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:F42"/>
@@ -6434,7 +6428,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002D6A4F"/>
+    <tabColor rgb="00C9B8B8"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:O30"/>
@@ -8165,7 +8159,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="002D6A4F"/>
+    <tabColor rgb="00C9B8B8"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:K103"/>
@@ -10812,7 +10806,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0040916C"/>
+    <tabColor rgb="00B2A0A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:G19"/>
@@ -11324,7 +11318,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0052B788"/>
+    <tabColor rgb="00C9B8B8"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:N24"/>
@@ -11427,7 +11421,7 @@
     </row>
     <row r="3">
       <c r="A3" s="43" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="B3" s="45" t="n">
         <v>1375</v>
@@ -11475,7 +11469,7 @@
     </row>
     <row r="4">
       <c r="A4" s="47" t="n">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="B4" s="49" t="n">
         <v>1375</v>
@@ -11523,7 +11517,7 @@
     </row>
     <row r="5">
       <c r="A5" s="43" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
       <c r="B5" s="45" t="n">
         <v>1375</v>
@@ -11571,7 +11565,7 @@
     </row>
     <row r="6">
       <c r="A6" s="47" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="B6" s="49" t="n">
         <v>1375</v>
@@ -11619,7 +11613,7 @@
     </row>
     <row r="7">
       <c r="A7" s="43" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
       <c r="B7" s="45" t="n">
         <v>1375</v>
@@ -11667,7 +11661,7 @@
     </row>
     <row r="8">
       <c r="A8" s="47" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="B8" s="49" t="n">
         <v>1375</v>
@@ -11715,7 +11709,7 @@
     </row>
     <row r="9">
       <c r="A9" s="43" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B9" s="45" t="n">
         <v>1375</v>
@@ -11763,7 +11757,7 @@
     </row>
     <row r="10">
       <c r="A10" s="47" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="B10" s="49" t="n">
         <v>1375</v>
@@ -11811,7 +11805,7 @@
     </row>
     <row r="11">
       <c r="A11" s="43" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="B11" s="45" t="n">
         <v>1375</v>
@@ -11859,7 +11853,7 @@
     </row>
     <row r="12">
       <c r="A12" s="47" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="B12" s="49" t="n">
         <v>1375</v>
@@ -11907,7 +11901,7 @@
     </row>
     <row r="13">
       <c r="A13" s="43" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="B13" s="45" t="n">
         <v>1375</v>
@@ -11955,7 +11949,7 @@
     </row>
     <row r="14">
       <c r="A14" s="47" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="B14" s="49" t="n">
         <v>1375</v>
@@ -12267,7 +12261,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="0074C69D"/>
+    <tabColor rgb="00D4EDEA"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:D16"/>
@@ -12536,7 +12530,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00E63946"/>
+    <tabColor rgb="00D4756B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:M525"/>
@@ -27281,7 +27275,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00F4A261"/>
+    <tabColor rgb="00C9A84C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:K131"/>

</xml_diff>